<commit_message>
Anomalies SF1-RPP2 — 25/09/2026
</commit_message>
<xml_diff>
--- a/presentation/SF1-RPP2/anomalies.xlsx
+++ b/presentation/SF1-RPP2/anomalies.xlsx
@@ -17,7 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -66,11 +69,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -436,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1"/>
+  <dimension ref="A1:U2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -456,9 +460,10 @@
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="27" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="15" customWidth="1" min="19" max="19"/>
-    <col width="22" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="15" customWidth="1" min="20" max="20"/>
+    <col width="22" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -549,17 +554,107 @@
       </c>
       <c r="R1" s="1" t="inlineStr">
         <is>
+          <t>Nb anomalies</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
           <t>Anomalie</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Responsable</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Action recommandée</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>11898787</v>
+      </c>
+      <c r="B2" t="n">
+        <v>4001089083</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Réparation collet Vanne pneumatique ACP</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>OR004001089083</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>SF01-PP-PP02-0CAP3Y-CA54ST-CIRC-CIRCUIT</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>CIRCUIT</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>SF1-RPP2</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>GM9</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>SF01</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>CRÉÉ CCRP DANP PART</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>ATER</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Y.ESSMAOUI</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="n">
+        <v>46292</v>
+      </c>
+      <c r="Q2" s="2" t="n">
+        <v>46043</v>
+      </c>
+      <c r="R2" t="n">
+        <v>1</v>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>OT préparation &gt;3 mois</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>Préparateur Méthodes</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>Traiter d'urgence les blocages de longue durée (&gt;3 mois) ou annuler les OT devenus sans objet.</t>
         </is>
       </c>
     </row>

</xml_diff>